<commit_message>
Correção de dados incompletos
O código filtrava apenas ELEITOS, omitindo ELEITOS POR MEDIA e ELEITOS POR QP.

Relatório em PDF atualizado.
</commit_message>
<xml_diff>
--- a/dados_tratados/resultado_salesopolis.xlsx
+++ b/dados_tratados/resultado_salesopolis.xlsx
@@ -5,26 +5,30 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6aa46f3471333097/Documentos/eleicoes_salesopolis/dados_tratados/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6aa46f3471333097/Documentos/analise-eleitoral-salesopolis/dados_tratados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_80507D5DA9BDB8338F024B6E18CFACC761164A40" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33AC5CEB-FF65-46CD-AE2C-628BE0BA9D81}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_D9D23C5FACF5B43CBF335916FCD1BC6A5994BA27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3326564-F876-4965-ACB4-2F7ED06E0254}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Matriz_Votos_Salesopolis" sheetId="1" r:id="rId1"/>
     <sheet name="Votos_Espectro_%" sheetId="2" r:id="rId2"/>
-    <sheet name="Eleitos_Espectro_%" sheetId="3" r:id="rId3"/>
+    <sheet name="Eleitos_Por_Partido" sheetId="3" r:id="rId3"/>
     <sheet name="Candidatos_Por_Partido" sheetId="4" r:id="rId4"/>
     <sheet name="Candidatos_Espectro_%" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Candidatos_Por_Partido!$A$1:$F$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Eleitos_Por_Partido!$A$1:$F$60</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="144">
   <si>
     <t>ESPECTRO</t>
   </si>
@@ -446,6 +450,12 @@
     <t>Presidente</t>
   </si>
   <si>
+    <t>QTD_ELEITOS</t>
+  </si>
+  <si>
+    <t>%_ELEITOS</t>
+  </si>
+  <si>
     <t>QTD_CANDIDATOS</t>
   </si>
   <si>
@@ -792,9 +802,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BR58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="29" max="29" width="22.109375" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:70" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -13933,10 +13940,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>131</v>
       </c>
@@ -13944,212 +13951,1207 @@
         <v>132</v>
       </c>
       <c r="C1" t="s">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
+        <v>140</v>
+      </c>
+      <c r="F1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>1996</v>
       </c>
       <c r="B2" t="s">
         <v>135</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>100</v>
       </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1996</v>
+      </c>
       <c r="B3" t="s">
         <v>136</v>
       </c>
-      <c r="C3">
-        <v>100</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>44.444444444444443</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>2000</v>
+        <v>1996</v>
       </c>
       <c r="B4" t="s">
         <v>136</v>
       </c>
-      <c r="C4">
-        <v>80</v>
-      </c>
-      <c r="D4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>2004</v>
+      <c r="C4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1996</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C5">
-        <v>100</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
+        <v>136</v>
+      </c>
+      <c r="C5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>11.111111111111111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1996</v>
+      </c>
       <c r="B6" t="s">
         <v>136</v>
       </c>
-      <c r="C6">
-        <v>100</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
-        <v>2008</v>
+      <c r="C6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2000</v>
       </c>
       <c r="B7" t="s">
         <v>135</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
         <v>100</v>
       </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2000</v>
+      </c>
       <c r="B8" t="s">
         <v>136</v>
       </c>
-      <c r="C8">
-        <v>66.666666666666657</v>
-      </c>
-      <c r="D8">
-        <v>33.333333333333329</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>2012</v>
+      <c r="C8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>11.111111111111111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>2000</v>
       </c>
       <c r="B9" t="s">
-        <v>135</v>
-      </c>
-      <c r="C9">
-        <v>100</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="1"/>
+        <v>136</v>
+      </c>
+      <c r="C9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>2000</v>
+      </c>
       <c r="B10" t="s">
         <v>136</v>
       </c>
-      <c r="C10">
-        <v>100</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>92</v>
+      </c>
+      <c r="D10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>2016</v>
+        <v>2000</v>
       </c>
       <c r="B11" t="s">
         <v>136</v>
       </c>
-      <c r="C11">
-        <v>88.888888888888886</v>
-      </c>
-      <c r="D11">
+      <c r="C11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>2000</v>
+      </c>
+      <c r="B12" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" t="s">
+        <v>96</v>
+      </c>
+      <c r="D12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
         <v>11.111111111111111</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
-        <v>2020</v>
-      </c>
-      <c r="B12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C12">
-        <v>100</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>2000</v>
+      </c>
       <c r="B13" t="s">
         <v>136</v>
       </c>
-      <c r="C13">
-        <v>100</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
-        <v>2024</v>
+      <c r="C13" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>11.111111111111111</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>2004</v>
       </c>
       <c r="B14" t="s">
         <v>135</v>
       </c>
-      <c r="C14">
+      <c r="C14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
         <v>100</v>
       </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2004</v>
+      </c>
       <c r="B15" t="s">
         <v>136</v>
       </c>
-      <c r="C15">
+      <c r="C15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>11.111111111111111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>2004</v>
+      </c>
+      <c r="B16" t="s">
+        <v>136</v>
+      </c>
+      <c r="C16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>33.333333333333329</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>2004</v>
+      </c>
+      <c r="B17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>11.111111111111111</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2004</v>
+      </c>
+      <c r="B18" t="s">
+        <v>136</v>
+      </c>
+      <c r="C18" t="s">
+        <v>96</v>
+      </c>
+      <c r="D18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2004</v>
+      </c>
+      <c r="B19" t="s">
+        <v>136</v>
+      </c>
+      <c r="C19" t="s">
         <v>100</v>
       </c>
-      <c r="D15">
-        <v>0</v>
+      <c r="D19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19">
+        <v>2</v>
+      </c>
+      <c r="F19">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>2008</v>
+      </c>
+      <c r="B20" t="s">
+        <v>135</v>
+      </c>
+      <c r="C20" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>2008</v>
+      </c>
+      <c r="B21" t="s">
+        <v>136</v>
+      </c>
+      <c r="C21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21">
+        <v>2</v>
+      </c>
+      <c r="F21">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>2008</v>
+      </c>
+      <c r="B22" t="s">
+        <v>136</v>
+      </c>
+      <c r="C22" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
+      <c r="F22">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2008</v>
+      </c>
+      <c r="B23" t="s">
+        <v>136</v>
+      </c>
+      <c r="C23" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" t="s">
+        <v>70</v>
+      </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
+      <c r="F23">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2008</v>
+      </c>
+      <c r="B24" t="s">
+        <v>136</v>
+      </c>
+      <c r="C24" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" t="s">
+        <v>105</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>11.111111111111111</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2008</v>
+      </c>
+      <c r="B25" t="s">
+        <v>136</v>
+      </c>
+      <c r="C25" t="s">
+        <v>98</v>
+      </c>
+      <c r="D25" t="s">
+        <v>70</v>
+      </c>
+      <c r="E25">
+        <v>2</v>
+      </c>
+      <c r="F25">
+        <v>22.222222222222221</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>2012</v>
+      </c>
+      <c r="B26" t="s">
+        <v>135</v>
+      </c>
+      <c r="C26" t="s">
+        <v>83</v>
+      </c>
+      <c r="D26" t="s">
+        <v>70</v>
+      </c>
+      <c r="E26">
+        <v>2</v>
+      </c>
+      <c r="F26">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>2012</v>
+      </c>
+      <c r="B27" t="s">
+        <v>136</v>
+      </c>
+      <c r="C27" t="s">
+        <v>73</v>
+      </c>
+      <c r="D27" t="s">
+        <v>70</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>2012</v>
+      </c>
+      <c r="B28" t="s">
+        <v>136</v>
+      </c>
+      <c r="C28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D28" t="s">
+        <v>70</v>
+      </c>
+      <c r="E28">
+        <v>2</v>
+      </c>
+      <c r="F28">
+        <v>18.18181818181818</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>2012</v>
+      </c>
+      <c r="B29" t="s">
+        <v>136</v>
+      </c>
+      <c r="C29" t="s">
+        <v>83</v>
+      </c>
+      <c r="D29" t="s">
+        <v>70</v>
+      </c>
+      <c r="E29">
+        <v>3</v>
+      </c>
+      <c r="F29">
+        <v>27.27272727272727</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>2012</v>
+      </c>
+      <c r="B30" t="s">
+        <v>136</v>
+      </c>
+      <c r="C30" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" t="s">
+        <v>70</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>2012</v>
+      </c>
+      <c r="B31" t="s">
+        <v>136</v>
+      </c>
+      <c r="C31" t="s">
+        <v>96</v>
+      </c>
+      <c r="D31" t="s">
+        <v>70</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>2012</v>
+      </c>
+      <c r="B32" t="s">
+        <v>136</v>
+      </c>
+      <c r="C32" t="s">
+        <v>113</v>
+      </c>
+      <c r="D32" t="s">
+        <v>105</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>2012</v>
+      </c>
+      <c r="B33" t="s">
+        <v>136</v>
+      </c>
+      <c r="C33" t="s">
+        <v>98</v>
+      </c>
+      <c r="D33" t="s">
+        <v>70</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>2012</v>
+      </c>
+      <c r="B34" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" t="s">
+        <v>70</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>2016</v>
+      </c>
+      <c r="B35" t="s">
+        <v>135</v>
+      </c>
+      <c r="C35" t="s">
+        <v>83</v>
+      </c>
+      <c r="D35" t="s">
+        <v>70</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>2016</v>
+      </c>
+      <c r="B36" t="s">
+        <v>135</v>
+      </c>
+      <c r="C36" t="s">
+        <v>100</v>
+      </c>
+      <c r="D36" t="s">
+        <v>70</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>2016</v>
+      </c>
+      <c r="B37" t="s">
+        <v>136</v>
+      </c>
+      <c r="C37" t="s">
+        <v>73</v>
+      </c>
+      <c r="D37" t="s">
+        <v>70</v>
+      </c>
+      <c r="E37">
+        <v>1</v>
+      </c>
+      <c r="F37">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>2016</v>
+      </c>
+      <c r="B38" t="s">
+        <v>136</v>
+      </c>
+      <c r="C38" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" t="s">
+        <v>70</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>18.18181818181818</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>2016</v>
+      </c>
+      <c r="B39" t="s">
+        <v>136</v>
+      </c>
+      <c r="C39" t="s">
+        <v>81</v>
+      </c>
+      <c r="D39" t="s">
+        <v>70</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>2016</v>
+      </c>
+      <c r="B40" t="s">
+        <v>136</v>
+      </c>
+      <c r="C40" t="s">
+        <v>83</v>
+      </c>
+      <c r="D40" t="s">
+        <v>70</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <v>18.18181818181818</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>2016</v>
+      </c>
+      <c r="B41" t="s">
+        <v>136</v>
+      </c>
+      <c r="C41" t="s">
+        <v>110</v>
+      </c>
+      <c r="D41" t="s">
+        <v>105</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>2016</v>
+      </c>
+      <c r="B42" t="s">
+        <v>136</v>
+      </c>
+      <c r="C42" t="s">
+        <v>95</v>
+      </c>
+      <c r="D42" t="s">
+        <v>70</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42">
+        <v>18.18181818181818</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>2016</v>
+      </c>
+      <c r="B43" t="s">
+        <v>136</v>
+      </c>
+      <c r="C43" t="s">
+        <v>96</v>
+      </c>
+      <c r="D43" t="s">
+        <v>70</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>2016</v>
+      </c>
+      <c r="B44" t="s">
+        <v>136</v>
+      </c>
+      <c r="C44" t="s">
+        <v>98</v>
+      </c>
+      <c r="D44" t="s">
+        <v>70</v>
+      </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
+      <c r="F44">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>2020</v>
+      </c>
+      <c r="B45" t="s">
+        <v>135</v>
+      </c>
+      <c r="C45" t="s">
+        <v>83</v>
+      </c>
+      <c r="D45" t="s">
+        <v>70</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
+      <c r="F45">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>2020</v>
+      </c>
+      <c r="B46" t="s">
+        <v>135</v>
+      </c>
+      <c r="C46" t="s">
+        <v>95</v>
+      </c>
+      <c r="D46" t="s">
+        <v>70</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>2020</v>
+      </c>
+      <c r="B47" t="s">
+        <v>136</v>
+      </c>
+      <c r="C47" t="s">
+        <v>72</v>
+      </c>
+      <c r="D47" t="s">
+        <v>70</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>2020</v>
+      </c>
+      <c r="B48" t="s">
+        <v>136</v>
+      </c>
+      <c r="C48" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48" t="s">
+        <v>70</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>2020</v>
+      </c>
+      <c r="B49" t="s">
+        <v>136</v>
+      </c>
+      <c r="C49" t="s">
+        <v>81</v>
+      </c>
+      <c r="D49" t="s">
+        <v>70</v>
+      </c>
+      <c r="E49">
+        <v>2</v>
+      </c>
+      <c r="F49">
+        <v>18.18181818181818</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>2020</v>
+      </c>
+      <c r="B50" t="s">
+        <v>136</v>
+      </c>
+      <c r="C50" t="s">
+        <v>83</v>
+      </c>
+      <c r="D50" t="s">
+        <v>70</v>
+      </c>
+      <c r="E50">
+        <v>4</v>
+      </c>
+      <c r="F50">
+        <v>36.363636363636367</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>2020</v>
+      </c>
+      <c r="B51" t="s">
+        <v>136</v>
+      </c>
+      <c r="C51" t="s">
+        <v>95</v>
+      </c>
+      <c r="D51" t="s">
+        <v>70</v>
+      </c>
+      <c r="E51">
+        <v>2</v>
+      </c>
+      <c r="F51">
+        <v>18.18181818181818</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>2020</v>
+      </c>
+      <c r="B52" t="s">
+        <v>136</v>
+      </c>
+      <c r="C52" t="s">
+        <v>96</v>
+      </c>
+      <c r="D52" t="s">
+        <v>70</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="F52">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>2024</v>
+      </c>
+      <c r="B53" t="s">
+        <v>135</v>
+      </c>
+      <c r="C53" t="s">
+        <v>86</v>
+      </c>
+      <c r="D53" t="s">
+        <v>70</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+      <c r="F53">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>2024</v>
+      </c>
+      <c r="B54" t="s">
+        <v>135</v>
+      </c>
+      <c r="C54" t="s">
+        <v>103</v>
+      </c>
+      <c r="D54" t="s">
+        <v>70</v>
+      </c>
+      <c r="E54">
+        <v>1</v>
+      </c>
+      <c r="F54">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>2024</v>
+      </c>
+      <c r="B55" t="s">
+        <v>136</v>
+      </c>
+      <c r="C55" t="s">
+        <v>74</v>
+      </c>
+      <c r="D55" t="s">
+        <v>70</v>
+      </c>
+      <c r="E55">
+        <v>2</v>
+      </c>
+      <c r="F55">
+        <v>18.18181818181818</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>2024</v>
+      </c>
+      <c r="B56" t="s">
+        <v>136</v>
+      </c>
+      <c r="C56" t="s">
+        <v>76</v>
+      </c>
+      <c r="D56" t="s">
+        <v>70</v>
+      </c>
+      <c r="E56">
+        <v>1</v>
+      </c>
+      <c r="F56">
+        <v>9.0909090909090917</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>2024</v>
+      </c>
+      <c r="B57" t="s">
+        <v>136</v>
+      </c>
+      <c r="C57" t="s">
+        <v>83</v>
+      </c>
+      <c r="D57" t="s">
+        <v>70</v>
+      </c>
+      <c r="E57">
+        <v>2</v>
+      </c>
+      <c r="F57">
+        <v>18.18181818181818</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>2024</v>
+      </c>
+      <c r="B58" t="s">
+        <v>136</v>
+      </c>
+      <c r="C58" t="s">
+        <v>84</v>
+      </c>
+      <c r="D58" t="s">
+        <v>70</v>
+      </c>
+      <c r="E58">
+        <v>2</v>
+      </c>
+      <c r="F58">
+        <v>18.18181818181818</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>2024</v>
+      </c>
+      <c r="B59" t="s">
+        <v>136</v>
+      </c>
+      <c r="C59" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59" t="s">
+        <v>70</v>
+      </c>
+      <c r="E59">
+        <v>3</v>
+      </c>
+      <c r="F59">
+        <v>27.27272727272727</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>2024</v>
+      </c>
+      <c r="B60" t="s">
+        <v>136</v>
+      </c>
+      <c r="C60" t="s">
+        <v>95</v>
+      </c>
+      <c r="D60" t="s">
+        <v>70</v>
+      </c>
+      <c r="E60">
+        <v>1</v>
+      </c>
+      <c r="F60">
+        <v>9.0909090909090917</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A2:A3"/>
-  </mergeCells>
+  <autoFilter ref="A1:F60" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F165"/>
+  <dimension ref="A1:F159"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -14166,10 +15168,10 @@
         <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -14506,10 +15508,10 @@
         <v>70</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18">
-        <v>20</v>
+        <v>33.333333333333329</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -14520,16 +15522,16 @@
         <v>135</v>
       </c>
       <c r="C19" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="D19" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="F19">
-        <v>20</v>
+        <v>16.666666666666661</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -14540,16 +15542,16 @@
         <v>135</v>
       </c>
       <c r="C20" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="D20" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20">
-        <v>40</v>
+        <v>16.666666666666661</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -14560,7 +15562,7 @@
         <v>135</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D21" t="s">
         <v>70</v>
@@ -14569,7 +15571,7 @@
         <v>1</v>
       </c>
       <c r="F21">
-        <v>20</v>
+        <v>16.666666666666661</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -14577,19 +15579,19 @@
         <v>2000</v>
       </c>
       <c r="B22" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C22" t="s">
-        <v>73</v>
+        <v>100</v>
       </c>
       <c r="D22" t="s">
         <v>70</v>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22">
-        <v>2.8985507246376812</v>
+        <v>16.666666666666661</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -14600,16 +15602,16 @@
         <v>136</v>
       </c>
       <c r="C23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D23" t="s">
         <v>70</v>
       </c>
       <c r="E23">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F23">
-        <v>15.942028985507241</v>
+        <v>10.8433734939759</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -14620,16 +15622,16 @@
         <v>136</v>
       </c>
       <c r="C24" t="s">
-        <v>106</v>
+        <v>76</v>
       </c>
       <c r="D24" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E24">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="F24">
-        <v>1.449275362318841</v>
+        <v>15.66265060240964</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -14646,10 +15648,10 @@
         <v>70</v>
       </c>
       <c r="E25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F25">
-        <v>5.7971014492753623</v>
+        <v>2.4096385542168681</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -14666,10 +15668,10 @@
         <v>70</v>
       </c>
       <c r="E26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F26">
-        <v>8.695652173913043</v>
+        <v>8.4337349397590362</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -14680,16 +15682,16 @@
         <v>136</v>
       </c>
       <c r="C27" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D27" t="s">
         <v>70</v>
       </c>
       <c r="E27">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F27">
-        <v>2.8985507246376812</v>
+        <v>9.6385542168674707</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -14700,16 +15702,16 @@
         <v>136</v>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="D28" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E28">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F28">
-        <v>7.2463768115942031</v>
+        <v>10.8433734939759</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -14720,16 +15722,16 @@
         <v>136</v>
       </c>
       <c r="C29" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="D29" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E29">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F29">
-        <v>14.49275362318841</v>
+        <v>3.6144578313253009</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -14740,16 +15742,16 @@
         <v>136</v>
       </c>
       <c r="C30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D30" t="s">
         <v>70</v>
       </c>
       <c r="E30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F30">
-        <v>7.2463768115942031</v>
+        <v>4.8192771084337354</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -14760,16 +15762,16 @@
         <v>136</v>
       </c>
       <c r="C31" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D31" t="s">
         <v>70</v>
       </c>
       <c r="E31">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F31">
-        <v>4.3478260869565224</v>
+        <v>10.8433734939759</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -14780,16 +15782,16 @@
         <v>136</v>
       </c>
       <c r="C32" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="D32" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F32">
-        <v>7.2463768115942031</v>
+        <v>2.4096385542168681</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
@@ -14800,16 +15802,16 @@
         <v>136</v>
       </c>
       <c r="C33" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="D33" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F33">
-        <v>1.449275362318841</v>
+        <v>7.2289156626506017</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -14820,36 +15822,36 @@
         <v>136</v>
       </c>
       <c r="C34" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D34" t="s">
         <v>70</v>
       </c>
       <c r="E34">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F34">
-        <v>11.594202898550719</v>
+        <v>13.253012048192771</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>2000</v>
+        <v>2004</v>
       </c>
       <c r="B35" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C35" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="D35" t="s">
         <v>70</v>
       </c>
       <c r="E35">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F35">
-        <v>8.695652173913043</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
@@ -14860,16 +15862,16 @@
         <v>135</v>
       </c>
       <c r="C36" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D36" t="s">
         <v>70</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36">
-        <v>7.6923076923076934</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -14880,16 +15882,16 @@
         <v>135</v>
       </c>
       <c r="C37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D37" t="s">
         <v>70</v>
       </c>
       <c r="E37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37">
-        <v>7.6923076923076934</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -14900,16 +15902,16 @@
         <v>135</v>
       </c>
       <c r="C38" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D38" t="s">
         <v>70</v>
       </c>
       <c r="E38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F38">
-        <v>7.6923076923076934</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -14920,7 +15922,7 @@
         <v>135</v>
       </c>
       <c r="C39" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D39" t="s">
         <v>70</v>
@@ -14929,7 +15931,7 @@
         <v>2</v>
       </c>
       <c r="F39">
-        <v>15.38461538461539</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -14940,16 +15942,16 @@
         <v>135</v>
       </c>
       <c r="C40" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D40" t="s">
         <v>70</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40">
-        <v>15.38461538461539</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
@@ -14960,7 +15962,7 @@
         <v>135</v>
       </c>
       <c r="C41" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="D41" t="s">
         <v>70</v>
@@ -14969,7 +15971,7 @@
         <v>1</v>
       </c>
       <c r="F41">
-        <v>7.6923076923076934</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -14980,16 +15982,16 @@
         <v>135</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="D42" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42">
-        <v>7.6923076923076934</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -15000,16 +16002,16 @@
         <v>135</v>
       </c>
       <c r="C43" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="D43" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43">
-        <v>7.6923076923076934</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -15020,16 +16022,16 @@
         <v>135</v>
       </c>
       <c r="C44" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D44" t="s">
         <v>70</v>
       </c>
       <c r="E44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44">
-        <v>15.38461538461539</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -15037,19 +16039,19 @@
         <v>2004</v>
       </c>
       <c r="B45" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C45" t="s">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="D45" t="s">
         <v>70</v>
       </c>
       <c r="E45">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F45">
-        <v>7.6923076923076934</v>
+        <v>2.4539877300613502</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -15060,16 +16062,16 @@
         <v>136</v>
       </c>
       <c r="C46" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D46" t="s">
         <v>70</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F46">
-        <v>0.98039215686274506</v>
+        <v>5.5214723926380369</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -15080,16 +16082,16 @@
         <v>136</v>
       </c>
       <c r="C47" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D47" t="s">
         <v>70</v>
       </c>
       <c r="E47">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F47">
-        <v>2.9411764705882351</v>
+        <v>2.4539877300613502</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -15100,16 +16102,16 @@
         <v>136</v>
       </c>
       <c r="C48" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D48" t="s">
         <v>70</v>
       </c>
       <c r="E48">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="F48">
-        <v>2.9411764705882351</v>
+        <v>6.7484662576687118</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -15120,16 +16122,16 @@
         <v>136</v>
       </c>
       <c r="C49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D49" t="s">
         <v>70</v>
       </c>
       <c r="E49">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F49">
-        <v>6.8627450980392162</v>
+        <v>6.1349693251533743</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -15140,16 +16142,16 @@
         <v>136</v>
       </c>
       <c r="C50" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="D50" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E50">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F50">
-        <v>4.9019607843137258</v>
+        <v>1.8404907975460121</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -15160,16 +16162,16 @@
         <v>136</v>
       </c>
       <c r="C51" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D51" t="s">
         <v>105</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F51">
-        <v>0.98039215686274506</v>
+        <v>1.2269938650306751</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -15180,16 +16182,16 @@
         <v>136</v>
       </c>
       <c r="C52" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="D52" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E52">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F52">
-        <v>1.9607843137254899</v>
+        <v>3.0674846625766872</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
@@ -15200,16 +16202,16 @@
         <v>136</v>
       </c>
       <c r="C53" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D53" t="s">
         <v>70</v>
       </c>
       <c r="E53">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F53">
-        <v>6.8627450980392162</v>
+        <v>7.3619631901840492</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
@@ -15220,16 +16222,16 @@
         <v>136</v>
       </c>
       <c r="C54" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D54" t="s">
         <v>70</v>
       </c>
       <c r="E54">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F54">
-        <v>8.8235294117647065</v>
+        <v>6.1349693251533743</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
@@ -15240,16 +16242,16 @@
         <v>136</v>
       </c>
       <c r="C55" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D55" t="s">
         <v>70</v>
       </c>
       <c r="E55">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F55">
-        <v>7.8431372549019596</v>
+        <v>2.4539877300613502</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
@@ -15260,16 +16262,16 @@
         <v>136</v>
       </c>
       <c r="C56" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D56" t="s">
         <v>70</v>
       </c>
       <c r="E56">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F56">
-        <v>2.9411764705882351</v>
+        <v>6.1349693251533743</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
@@ -15280,7 +16282,7 @@
         <v>136</v>
       </c>
       <c r="C57" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D57" t="s">
         <v>70</v>
@@ -15289,7 +16291,7 @@
         <v>4</v>
       </c>
       <c r="F57">
-        <v>3.9215686274509798</v>
+        <v>2.4539877300613502</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
@@ -15300,16 +16302,16 @@
         <v>136</v>
       </c>
       <c r="C58" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D58" t="s">
         <v>70</v>
       </c>
       <c r="E58">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F58">
-        <v>0.98039215686274506</v>
+        <v>2.4539877300613502</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
@@ -15320,16 +16322,16 @@
         <v>136</v>
       </c>
       <c r="C59" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="D59" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E59">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F59">
-        <v>0.98039215686274506</v>
+        <v>3.0674846625766872</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
@@ -15340,16 +16342,16 @@
         <v>136</v>
       </c>
       <c r="C60" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="D60" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E60">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F60">
-        <v>3.9215686274509798</v>
+        <v>6.1349693251533743</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
@@ -15360,16 +16362,16 @@
         <v>136</v>
       </c>
       <c r="C61" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D61" t="s">
         <v>70</v>
       </c>
       <c r="E61">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F61">
-        <v>5.8823529411764701</v>
+        <v>7.3619631901840492</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
@@ -15380,16 +16382,16 @@
         <v>136</v>
       </c>
       <c r="C62" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D62" t="s">
         <v>70</v>
       </c>
       <c r="E62">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F62">
-        <v>5.8823529411764701</v>
+        <v>2.4539877300613502</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
@@ -15400,16 +16402,16 @@
         <v>136</v>
       </c>
       <c r="C63" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="D63" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E63">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F63">
-        <v>1.9607843137254899</v>
+        <v>8.5889570552147241</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
@@ -15420,16 +16422,16 @@
         <v>136</v>
       </c>
       <c r="C64" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="D64" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E64">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F64">
-        <v>8.8235294117647065</v>
+        <v>9.2024539877300615</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
@@ -15440,36 +16442,36 @@
         <v>136</v>
       </c>
       <c r="C65" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D65" t="s">
         <v>70</v>
       </c>
       <c r="E65">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F65">
-        <v>11.76470588235294</v>
+        <v>6.7484662576687118</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>2004</v>
+        <v>2008</v>
       </c>
       <c r="B66" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C66" t="s">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="D66" t="s">
         <v>70</v>
       </c>
       <c r="E66">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F66">
-        <v>7.8431372549019596</v>
+        <v>16.666666666666661</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
@@ -15480,7 +16482,7 @@
         <v>135</v>
       </c>
       <c r="C67" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="D67" t="s">
         <v>70</v>
@@ -15489,7 +16491,7 @@
         <v>1</v>
       </c>
       <c r="F67">
-        <v>14.285714285714279</v>
+        <v>16.666666666666661</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
@@ -15500,16 +16502,16 @@
         <v>135</v>
       </c>
       <c r="C68" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="D68" t="s">
         <v>70</v>
       </c>
       <c r="E68">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F68">
-        <v>14.285714285714279</v>
+        <v>33.333333333333329</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
@@ -15520,7 +16522,7 @@
         <v>135</v>
       </c>
       <c r="C69" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="D69" t="s">
         <v>70</v>
@@ -15529,7 +16531,7 @@
         <v>1</v>
       </c>
       <c r="F69">
-        <v>14.285714285714279</v>
+        <v>16.666666666666661</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
@@ -15540,7 +16542,7 @@
         <v>135</v>
       </c>
       <c r="C70" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="D70" t="s">
         <v>70</v>
@@ -15549,7 +16551,7 @@
         <v>1</v>
       </c>
       <c r="F70">
-        <v>14.285714285714279</v>
+        <v>16.666666666666661</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
@@ -15557,10 +16559,10 @@
         <v>2008</v>
       </c>
       <c r="B71" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C71" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="D71" t="s">
         <v>70</v>
@@ -15569,7 +16571,7 @@
         <v>1</v>
       </c>
       <c r="F71">
-        <v>14.285714285714279</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
@@ -15577,19 +16579,19 @@
         <v>2008</v>
       </c>
       <c r="B72" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C72" t="s">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="D72" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E72">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F72">
-        <v>14.285714285714279</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
@@ -15597,19 +16599,19 @@
         <v>2008</v>
       </c>
       <c r="B73" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C73" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="D73" t="s">
         <v>70</v>
       </c>
       <c r="E73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F73">
-        <v>14.285714285714279</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
@@ -15620,16 +16622,16 @@
         <v>136</v>
       </c>
       <c r="C74" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D74" t="s">
         <v>70</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F74">
-        <v>3.0769230769230771</v>
+        <v>15</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
@@ -15640,16 +16642,16 @@
         <v>136</v>
       </c>
       <c r="C75" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="D75" t="s">
         <v>70</v>
       </c>
       <c r="E75">
+        <v>4</v>
+      </c>
+      <c r="F75">
         <v>5</v>
-      </c>
-      <c r="F75">
-        <v>7.6923076923076934</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
@@ -15660,16 +16662,16 @@
         <v>136</v>
       </c>
       <c r="C76" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="D76" t="s">
         <v>70</v>
       </c>
       <c r="E76">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F76">
-        <v>4.6153846153846159</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
@@ -15680,16 +16682,16 @@
         <v>136</v>
       </c>
       <c r="C77" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="D77" t="s">
         <v>70</v>
       </c>
       <c r="E77">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="F77">
-        <v>21.53846153846154</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
@@ -15700,16 +16702,16 @@
         <v>136</v>
       </c>
       <c r="C78" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="D78" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E78">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F78">
-        <v>7.6923076923076934</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
@@ -15720,16 +16722,16 @@
         <v>136</v>
       </c>
       <c r="C79" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="D79" t="s">
         <v>70</v>
       </c>
       <c r="E79">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="F79">
-        <v>7.6923076923076934</v>
+        <v>16.25</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
@@ -15740,16 +16742,16 @@
         <v>136</v>
       </c>
       <c r="C80" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="D80" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E80">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F80">
-        <v>3.0769230769230771</v>
+        <v>10</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
@@ -15760,16 +16762,16 @@
         <v>136</v>
       </c>
       <c r="C81" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="D81" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E81">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F81">
-        <v>6.1538461538461542</v>
+        <v>15</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
@@ -15780,76 +16782,76 @@
         <v>136</v>
       </c>
       <c r="C82" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D82" t="s">
         <v>70</v>
       </c>
       <c r="E82">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F82">
-        <v>12.30769230769231</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>2008</v>
+        <v>2012</v>
       </c>
       <c r="B83" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C83" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="D83" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E83">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F83">
-        <v>6.1538461538461542</v>
+        <v>25</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>2008</v>
+        <v>2012</v>
       </c>
       <c r="B84" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C84" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D84" t="s">
         <v>70</v>
       </c>
       <c r="E84">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F84">
-        <v>12.30769230769231</v>
+        <v>25</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85">
-        <v>2008</v>
+        <v>2012</v>
       </c>
       <c r="B85" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C85" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="D85" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E85">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F85">
-        <v>7.6923076923076934</v>
+        <v>25</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
@@ -15860,16 +16862,16 @@
         <v>135</v>
       </c>
       <c r="C86" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D86" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F86">
-        <v>14.285714285714279</v>
+        <v>25</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
@@ -15877,19 +16879,19 @@
         <v>2012</v>
       </c>
       <c r="B87" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C87" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="D87" t="s">
         <v>70</v>
       </c>
       <c r="E87">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F87">
-        <v>14.285714285714279</v>
+        <v>4.1322314049586781</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
@@ -15897,19 +16899,19 @@
         <v>2012</v>
       </c>
       <c r="B88" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C88" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="D88" t="s">
         <v>70</v>
       </c>
       <c r="E88">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F88">
-        <v>28.571428571428569</v>
+        <v>3.3057851239669418</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
@@ -15917,19 +16919,19 @@
         <v>2012</v>
       </c>
       <c r="B89" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C89" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="D89" t="s">
         <v>70</v>
       </c>
       <c r="E89">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F89">
-        <v>42.857142857142847</v>
+        <v>0.82644628099173556</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
@@ -15940,16 +16942,16 @@
         <v>136</v>
       </c>
       <c r="C90" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D90" t="s">
         <v>70</v>
       </c>
       <c r="E90">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F90">
-        <v>2.9702970297029698</v>
+        <v>8.2644628099173563</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
@@ -15960,16 +16962,16 @@
         <v>136</v>
       </c>
       <c r="C91" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D91" t="s">
         <v>70</v>
       </c>
       <c r="E91">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F91">
-        <v>1.98019801980198</v>
+        <v>2.4793388429752068</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
@@ -15980,16 +16982,16 @@
         <v>136</v>
       </c>
       <c r="C92" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="D92" t="s">
         <v>70</v>
       </c>
       <c r="E92">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="F92">
-        <v>2.9702970297029698</v>
+        <v>15.702479338842981</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
@@ -16000,16 +17002,16 @@
         <v>136</v>
       </c>
       <c r="C93" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="D93" t="s">
         <v>70</v>
       </c>
       <c r="E93">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F93">
-        <v>6.9306930693069324</v>
+        <v>2.4793388429752068</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
@@ -16020,16 +17022,16 @@
         <v>136</v>
       </c>
       <c r="C94" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D94" t="s">
         <v>105</v>
       </c>
       <c r="E94">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F94">
-        <v>3.9603960396039599</v>
+        <v>0.82644628099173556</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
@@ -16040,16 +17042,16 @@
         <v>136</v>
       </c>
       <c r="C95" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="D95" t="s">
         <v>70</v>
       </c>
       <c r="E95">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F95">
-        <v>1.98019801980198</v>
+        <v>9.9173553719008272</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
@@ -16060,16 +17062,16 @@
         <v>136</v>
       </c>
       <c r="C96" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="D96" t="s">
         <v>70</v>
       </c>
       <c r="E96">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F96">
-        <v>9.9009900990099009</v>
+        <v>7.4380165289256199</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
@@ -16080,16 +17082,16 @@
         <v>136</v>
       </c>
       <c r="C97" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="D97" t="s">
         <v>70</v>
       </c>
       <c r="E97">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F97">
-        <v>1.98019801980198</v>
+        <v>9.9173553719008272</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
@@ -16100,16 +17102,16 @@
         <v>136</v>
       </c>
       <c r="C98" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D98" t="s">
         <v>105</v>
       </c>
       <c r="E98">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="F98">
-        <v>1.98019801980198</v>
+        <v>14.049586776859501</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
@@ -16120,16 +17122,16 @@
         <v>136</v>
       </c>
       <c r="C99" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D99" t="s">
         <v>70</v>
       </c>
       <c r="E99">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F99">
-        <v>6.9306930693069324</v>
+        <v>9.0909090909090917</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
@@ -16140,96 +17142,96 @@
         <v>136</v>
       </c>
       <c r="C100" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D100" t="s">
         <v>70</v>
       </c>
       <c r="E100">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F100">
-        <v>10.89108910891089</v>
+        <v>11.5702479338843</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="B101" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C101" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="D101" t="s">
         <v>70</v>
       </c>
       <c r="E101">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F101">
-        <v>14.85148514851485</v>
+        <v>10</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="B102" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C102" t="s">
-        <v>113</v>
+        <v>76</v>
       </c>
       <c r="D102" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E102">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="F102">
-        <v>13.861386138613859</v>
+        <v>10</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="B103" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C103" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="D103" t="s">
         <v>70</v>
       </c>
       <c r="E103">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F103">
-        <v>5.9405940594059414</v>
+        <v>10</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104">
-        <v>2012</v>
+        <v>2016</v>
       </c>
       <c r="B104" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C104" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="D104" t="s">
         <v>70</v>
       </c>
       <c r="E104">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="F104">
-        <v>12.87128712871287</v>
+        <v>10</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
@@ -16240,16 +17242,16 @@
         <v>135</v>
       </c>
       <c r="C105" t="s">
-        <v>73</v>
+        <v>110</v>
       </c>
       <c r="D105" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E105">
         <v>1</v>
       </c>
       <c r="F105">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
@@ -16260,13 +17262,13 @@
         <v>135</v>
       </c>
       <c r="C106" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="D106" t="s">
         <v>70</v>
       </c>
       <c r="E106">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F106">
         <v>20</v>
@@ -16280,16 +17282,16 @@
         <v>135</v>
       </c>
       <c r="C107" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="D107" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E107">
         <v>1</v>
       </c>
       <c r="F107">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
@@ -16300,7 +17302,7 @@
         <v>135</v>
       </c>
       <c r="C108" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D108" t="s">
         <v>70</v>
@@ -16309,7 +17311,7 @@
         <v>1</v>
       </c>
       <c r="F108">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
@@ -16320,7 +17322,7 @@
         <v>135</v>
       </c>
       <c r="C109" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D109" t="s">
         <v>70</v>
@@ -16329,7 +17331,7 @@
         <v>1</v>
       </c>
       <c r="F109">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
@@ -16346,10 +17348,10 @@
         <v>70</v>
       </c>
       <c r="E110">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F110">
-        <v>3.125</v>
+        <v>1.666666666666667</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
@@ -16360,16 +17362,16 @@
         <v>136</v>
       </c>
       <c r="C111" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D111" t="s">
         <v>70</v>
       </c>
       <c r="E111">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F111">
-        <v>5.2083333333333339</v>
+        <v>6.666666666666667</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
@@ -16380,16 +17382,16 @@
         <v>136</v>
       </c>
       <c r="C112" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D112" t="s">
         <v>70</v>
       </c>
       <c r="E112">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F112">
-        <v>3.125</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
@@ -16400,16 +17402,16 @@
         <v>136</v>
       </c>
       <c r="C113" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D113" t="s">
         <v>70</v>
       </c>
       <c r="E113">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F113">
-        <v>7.291666666666667</v>
+        <v>11.66666666666667</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
@@ -16420,16 +17422,16 @@
         <v>136</v>
       </c>
       <c r="C114" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D114" t="s">
         <v>70</v>
       </c>
       <c r="E114">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F114">
-        <v>9.375</v>
+        <v>4.1666666666666661</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
@@ -16440,16 +17442,16 @@
         <v>136</v>
       </c>
       <c r="C115" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D115" t="s">
         <v>70</v>
       </c>
       <c r="E115">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F115">
-        <v>2.083333333333333</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
@@ -16460,16 +17462,16 @@
         <v>136</v>
       </c>
       <c r="C116" t="s">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="D116" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E116">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F116">
-        <v>1.041666666666667</v>
+        <v>1.666666666666667</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
@@ -16480,16 +17482,16 @@
         <v>136</v>
       </c>
       <c r="C117" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="D117" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E117">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F117">
-        <v>3.125</v>
+        <v>10</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
@@ -16500,7 +17502,7 @@
         <v>136</v>
       </c>
       <c r="C118" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="D118" t="s">
         <v>70</v>
@@ -16509,7 +17511,7 @@
         <v>1</v>
       </c>
       <c r="F118">
-        <v>1.041666666666667</v>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
@@ -16520,16 +17522,16 @@
         <v>136</v>
       </c>
       <c r="C119" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="D119" t="s">
         <v>70</v>
       </c>
       <c r="E119">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F119">
-        <v>9.375</v>
+        <v>14.16666666666667</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
@@ -16540,16 +17542,16 @@
         <v>136</v>
       </c>
       <c r="C120" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D120" t="s">
         <v>70</v>
       </c>
       <c r="E120">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F120">
-        <v>2.083333333333333</v>
+        <v>5.833333333333333</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
@@ -16560,16 +17562,16 @@
         <v>136</v>
       </c>
       <c r="C121" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="D121" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E121">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F121">
-        <v>2.083333333333333</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
@@ -16580,16 +17582,16 @@
         <v>136</v>
       </c>
       <c r="C122" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D122" t="s">
         <v>70</v>
       </c>
       <c r="E122">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F122">
-        <v>1.041666666666667</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
@@ -16600,16 +17602,16 @@
         <v>136</v>
       </c>
       <c r="C123" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="D123" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E123">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F123">
-        <v>9.375</v>
+        <v>1.666666666666667</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
@@ -16620,16 +17622,16 @@
         <v>136</v>
       </c>
       <c r="C124" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D124" t="s">
         <v>70</v>
       </c>
       <c r="E124">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F124">
-        <v>1.041666666666667</v>
+        <v>5.833333333333333</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
@@ -16640,16 +17642,16 @@
         <v>136</v>
       </c>
       <c r="C125" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D125" t="s">
         <v>70</v>
       </c>
       <c r="E125">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F125">
-        <v>8.3333333333333321</v>
+        <v>9.1666666666666661</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
@@ -16660,67 +17662,67 @@
         <v>136</v>
       </c>
       <c r="C126" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D126" t="s">
         <v>70</v>
       </c>
       <c r="E126">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F126">
-        <v>6.25</v>
+        <v>1.666666666666667</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="B127" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C127" t="s">
-        <v>113</v>
+        <v>75</v>
       </c>
       <c r="D127" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E127">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F127">
-        <v>3.125</v>
+        <v>20</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="B128" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C128" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="D128" t="s">
         <v>70</v>
       </c>
       <c r="E128">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F128">
-        <v>7.291666666666667</v>
+        <v>20</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="B129" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C129" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="D129" t="s">
         <v>70</v>
@@ -16729,58 +17731,58 @@
         <v>1</v>
       </c>
       <c r="F129">
-        <v>1.041666666666667</v>
+        <v>10</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="B130" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C130" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D130" t="s">
         <v>70</v>
       </c>
       <c r="E130">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F130">
-        <v>5.2083333333333339</v>
+        <v>20</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="B131" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C131" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D131" t="s">
         <v>70</v>
       </c>
       <c r="E131">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F131">
-        <v>6.25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132">
-        <v>2016</v>
+        <v>2020</v>
       </c>
       <c r="B132" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C132" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D132" t="s">
         <v>70</v>
@@ -16789,7 +17791,7 @@
         <v>2</v>
       </c>
       <c r="F132">
-        <v>2.083333333333333</v>
+        <v>20</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
@@ -16797,19 +17799,19 @@
         <v>2020</v>
       </c>
       <c r="B133" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C133" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D133" t="s">
         <v>70</v>
       </c>
       <c r="E133">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F133">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
@@ -16817,19 +17819,19 @@
         <v>2020</v>
       </c>
       <c r="B134" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C134" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="D134" t="s">
         <v>70</v>
       </c>
       <c r="E134">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="F134">
-        <v>20</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
@@ -16837,19 +17839,19 @@
         <v>2020</v>
       </c>
       <c r="B135" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C135" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D135" t="s">
         <v>70</v>
       </c>
       <c r="E135">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="F135">
-        <v>10</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
@@ -16857,19 +17859,19 @@
         <v>2020</v>
       </c>
       <c r="B136" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C136" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="D136" t="s">
         <v>70</v>
       </c>
       <c r="E136">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="F136">
-        <v>20</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
@@ -16877,7 +17879,7 @@
         <v>2020</v>
       </c>
       <c r="B137" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C137" t="s">
         <v>95</v>
@@ -16886,10 +17888,10 @@
         <v>70</v>
       </c>
       <c r="E137">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="F137">
-        <v>10</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
@@ -16897,7 +17899,7 @@
         <v>2020</v>
       </c>
       <c r="B138" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C138" t="s">
         <v>96</v>
@@ -16906,10 +17908,10 @@
         <v>70</v>
       </c>
       <c r="E138">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F138">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
@@ -16920,16 +17922,16 @@
         <v>136</v>
       </c>
       <c r="C139" t="s">
-        <v>72</v>
+        <v>113</v>
       </c>
       <c r="D139" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E139">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F139">
-        <v>12</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
@@ -16940,44 +17942,44 @@
         <v>136</v>
       </c>
       <c r="C140" t="s">
-        <v>75</v>
+        <v>101</v>
       </c>
       <c r="D140" t="s">
         <v>70</v>
       </c>
       <c r="E140">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F140">
-        <v>13.6</v>
+        <v>8.7999999999999989</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="B141" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C141" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D141" t="s">
         <v>70</v>
       </c>
       <c r="E141">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="F141">
-        <v>13.6</v>
+        <v>9.0909090909090917</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="B142" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C142" t="s">
         <v>83</v>
@@ -16986,58 +17988,58 @@
         <v>70</v>
       </c>
       <c r="E142">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="F142">
-        <v>13.6</v>
+        <v>27.27272727272727</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="B143" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C143" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="D143" t="s">
         <v>70</v>
       </c>
       <c r="E143">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="F143">
-        <v>13.6</v>
+        <v>9.0909090909090917</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="B144" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C144" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D144" t="s">
         <v>70</v>
       </c>
       <c r="E144">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F144">
-        <v>12</v>
+        <v>9.0909090909090917</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="B145" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C145" t="s">
         <v>113</v>
@@ -17046,30 +18048,30 @@
         <v>105</v>
       </c>
       <c r="E145">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F145">
-        <v>12.8</v>
+        <v>9.0909090909090917</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146">
-        <v>2020</v>
+        <v>2024</v>
       </c>
       <c r="B146" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C146" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D146" t="s">
         <v>70</v>
       </c>
       <c r="E146">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F146">
-        <v>8.7999999999999989</v>
+        <v>9.0909090909090917</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
@@ -17080,16 +18082,16 @@
         <v>135</v>
       </c>
       <c r="C147" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="D147" t="s">
         <v>70</v>
       </c>
       <c r="E147">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F147">
-        <v>9.0909090909090917</v>
+        <v>18.18181818181818</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
@@ -17100,16 +18102,16 @@
         <v>135</v>
       </c>
       <c r="C148" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="D148" t="s">
         <v>70</v>
       </c>
       <c r="E148">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F148">
-        <v>27.27272727272727</v>
+        <v>9.0909090909090917</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
@@ -17117,19 +18119,19 @@
         <v>2024</v>
       </c>
       <c r="B149" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C149" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="D149" t="s">
         <v>70</v>
       </c>
       <c r="E149">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F149">
-        <v>9.0909090909090917</v>
+        <v>10.90909090909091</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
@@ -17137,19 +18139,19 @@
         <v>2024</v>
       </c>
       <c r="B150" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C150" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="D150" t="s">
         <v>70</v>
       </c>
       <c r="E150">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F150">
-        <v>9.0909090909090917</v>
+        <v>10.90909090909091</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
@@ -17157,19 +18159,19 @@
         <v>2024</v>
       </c>
       <c r="B151" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C151" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="D151" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E151">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F151">
-        <v>9.0909090909090917</v>
+        <v>12.72727272727273</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
@@ -17177,19 +18179,19 @@
         <v>2024</v>
       </c>
       <c r="B152" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C152" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="D152" t="s">
         <v>70</v>
       </c>
       <c r="E152">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F152">
-        <v>9.0909090909090917</v>
+        <v>10.90909090909091</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
@@ -17197,19 +18199,19 @@
         <v>2024</v>
       </c>
       <c r="B153" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C153" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="D153" t="s">
         <v>70</v>
       </c>
       <c r="E153">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F153">
-        <v>18.18181818181818</v>
+        <v>9.0909090909090917</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
@@ -17217,19 +18219,19 @@
         <v>2024</v>
       </c>
       <c r="B154" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C154" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="D154" t="s">
         <v>70</v>
       </c>
       <c r="E154">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F154">
-        <v>9.0909090909090917</v>
+        <v>10.90909090909091</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
@@ -17240,7 +18242,7 @@
         <v>136</v>
       </c>
       <c r="C155" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="D155" t="s">
         <v>70</v>
@@ -17260,16 +18262,16 @@
         <v>136</v>
       </c>
       <c r="C156" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="D156" t="s">
         <v>70</v>
       </c>
       <c r="E156">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F156">
-        <v>10.90909090909091</v>
+        <v>10</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
@@ -17280,16 +18282,16 @@
         <v>136</v>
       </c>
       <c r="C157" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="D157" t="s">
-        <v>70</v>
+        <v>105</v>
       </c>
       <c r="E157">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F157">
-        <v>12.72727272727273</v>
+        <v>7.2727272727272716</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
@@ -17300,16 +18302,16 @@
         <v>136</v>
       </c>
       <c r="C158" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="D158" t="s">
         <v>70</v>
       </c>
       <c r="E158">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F158">
-        <v>10.90909090909091</v>
+        <v>3.6363636363636358</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
@@ -17320,139 +18322,20 @@
         <v>136</v>
       </c>
       <c r="C159" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="D159" t="s">
         <v>70</v>
       </c>
       <c r="E159">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F159">
-        <v>9.0909090909090917</v>
-      </c>
-    </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A160">
-        <v>2024</v>
-      </c>
-      <c r="B160" t="s">
-        <v>136</v>
-      </c>
-      <c r="C160" t="s">
-        <v>93</v>
-      </c>
-      <c r="D160" t="s">
-        <v>70</v>
-      </c>
-      <c r="E160">
-        <v>12</v>
-      </c>
-      <c r="F160">
-        <v>10.90909090909091</v>
-      </c>
-    </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A161">
-        <v>2024</v>
-      </c>
-      <c r="B161" t="s">
-        <v>136</v>
-      </c>
-      <c r="C161" t="s">
-        <v>95</v>
-      </c>
-      <c r="D161" t="s">
-        <v>70</v>
-      </c>
-      <c r="E161">
-        <v>12</v>
-      </c>
-      <c r="F161">
-        <v>10.90909090909091</v>
-      </c>
-    </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A162">
-        <v>2024</v>
-      </c>
-      <c r="B162" t="s">
-        <v>136</v>
-      </c>
-      <c r="C162" t="s">
-        <v>96</v>
-      </c>
-      <c r="D162" t="s">
-        <v>70</v>
-      </c>
-      <c r="E162">
-        <v>11</v>
-      </c>
-      <c r="F162">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A163">
-        <v>2024</v>
-      </c>
-      <c r="B163" t="s">
-        <v>136</v>
-      </c>
-      <c r="C163" t="s">
-        <v>113</v>
-      </c>
-      <c r="D163" t="s">
-        <v>105</v>
-      </c>
-      <c r="E163">
-        <v>8</v>
-      </c>
-      <c r="F163">
-        <v>7.2727272727272716</v>
-      </c>
-    </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A164">
-        <v>2024</v>
-      </c>
-      <c r="B164" t="s">
-        <v>136</v>
-      </c>
-      <c r="C164" t="s">
-        <v>100</v>
-      </c>
-      <c r="D164" t="s">
-        <v>70</v>
-      </c>
-      <c r="E164">
-        <v>4</v>
-      </c>
-      <c r="F164">
-        <v>3.6363636363636358</v>
-      </c>
-    </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A165">
-        <v>2024</v>
-      </c>
-      <c r="B165" t="s">
-        <v>136</v>
-      </c>
-      <c r="C165" t="s">
-        <v>102</v>
-      </c>
-      <c r="D165" t="s">
-        <v>70</v>
-      </c>
-      <c r="E165">
-        <v>3</v>
-      </c>
-      <c r="F165">
         <v>2.7272727272727271</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F159" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17510,10 +18393,10 @@
         <v>135</v>
       </c>
       <c r="C4">
-        <v>60</v>
+        <v>83.333333333333343</v>
       </c>
       <c r="D4">
-        <v>40</v>
+        <v>16.666666666666661</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -17522,10 +18405,10 @@
         <v>136</v>
       </c>
       <c r="C5">
-        <v>82.608695652173907</v>
+        <v>86.746987951807228</v>
       </c>
       <c r="D5">
-        <v>17.39130434782609</v>
+        <v>13.253012048192771</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -17536,10 +18419,10 @@
         <v>135</v>
       </c>
       <c r="C6">
-        <v>92.307692307692307</v>
+        <v>87.5</v>
       </c>
       <c r="D6">
-        <v>7.6923076923076934</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -17548,10 +18431,10 @@
         <v>136</v>
       </c>
       <c r="C7">
-        <v>84.313725490196077</v>
+        <v>85.276073619631902</v>
       </c>
       <c r="D7">
-        <v>15.686274509803919</v>
+        <v>14.7239263803681</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -17562,10 +18445,10 @@
         <v>135</v>
       </c>
       <c r="C8">
-        <v>85.714285714285708</v>
+        <v>100</v>
       </c>
       <c r="D8">
-        <v>14.285714285714279</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -17574,10 +18457,10 @@
         <v>136</v>
       </c>
       <c r="C9">
-        <v>87.692307692307693</v>
+        <v>86.25</v>
       </c>
       <c r="D9">
-        <v>12.30769230769231</v>
+        <v>13.75</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -17588,10 +18471,10 @@
         <v>135</v>
       </c>
       <c r="C10">
-        <v>85.714285714285708</v>
+        <v>75</v>
       </c>
       <c r="D10">
-        <v>14.285714285714279</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -17600,10 +18483,10 @@
         <v>136</v>
       </c>
       <c r="C11">
-        <v>80.198019801980209</v>
+        <v>85.123966942148769</v>
       </c>
       <c r="D11">
-        <v>19.801980198019798</v>
+        <v>14.87603305785124</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -17614,10 +18497,10 @@
         <v>135</v>
       </c>
       <c r="C12">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="D12">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -17626,10 +18509,10 @@
         <v>136</v>
       </c>
       <c r="C13">
-        <v>86.458333333333343</v>
+        <v>87.5</v>
       </c>
       <c r="D13">
-        <v>13.54166666666667</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>